<commit_message>
little ajustes tabela de dados
</commit_message>
<xml_diff>
--- a/data/DiagnosticoTPLC.xlsx
+++ b/data/DiagnosticoTPLC.xlsx
@@ -1,12 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pc\OneDrive\Documentos\D.comercial\dashboard streamlit\app\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A240189-B90A-42F5-89BC-74FFA5333D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Página1" sheetId="1" r:id="rId5"/>
+    <sheet name="Página1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -601,9 +615,6 @@
     <t>1.501,00 A 2.000,00</t>
   </si>
   <si>
-    <t>REDE DE ENSEADA:ARRASTO;TARRAFA;LINHA E ANZOL</t>
-  </si>
-  <si>
     <t>15 A 24 HORAS</t>
   </si>
   <si>
@@ -767,20 +778,24 @@
   </si>
   <si>
     <t>INDENIZACOES</t>
+  </si>
+  <si>
+    <t>REDE DE ENSEADA;ARRASTO;TARRAFA;LINHA E ANZOL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -791,76 +806,43 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -877,20 +859,48 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Página1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Página1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -898,56 +908,56 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AO35" displayName="Tabela_1" name="Tabela_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela_1" displayName="Tabela_1" ref="A1:AO35">
   <tableColumns count="41">
-    <tableColumn name="ID" id="1"/>
-    <tableColumn name="Nome" id="2"/>
-    <tableColumn name="Comunidade" id="3"/>
-    <tableColumn name="Genero" id="4"/>
-    <tableColumn name="Idade" id="5"/>
-    <tableColumn name="Estado_civil" id="6"/>
-    <tableColumn name="Contato" id="7"/>
-    <tableColumn name="Numero_dependentes_renda" id="8"/>
-    <tableColumn name="Familia_escolaridade" id="9"/>
-    <tableColumn name="Familia_faixa_etaria" id="10"/>
-    <tableColumn name="Renda_mensal_total_familia" id="11"/>
-    <tableColumn name="Renda_origem" id="12"/>
-    <tableColumn name="Tipo_pesca" id="13"/>
-    <tableColumn name="Tempo_pesca(anos)" id="14"/>
-    <tableColumn name="Arte_pesca" id="15"/>
-    <tableColumn name="Duracao_pescaria" id="16"/>
-    <tableColumn name="Frequencia_pescaria" id="17"/>
-    <tableColumn name="Numero_tripulantes" id="18"/>
-    <tableColumn name="Pesca_defeso" id="19"/>
-    <tableColumn name="Seguro_defeso" id="20"/>
-    <tableColumn name="Embarcacao_propria" id="21"/>
-    <tableColumn name="Tipo_embarcaçao" id="22"/>
-    <tableColumn name="Porte_embarcacao" id="23"/>
-    <tableColumn name="Tipo_propulsao" id="24"/>
-    <tableColumn name="Dias_sem_reabastecer" id="25"/>
-    <tableColumn name="Titularidade" id="26"/>
-    <tableColumn name="Onde_pesca" id="27"/>
-    <tableColumn name="Local_saida" id="28"/>
-    <tableColumn name="Local_desenbarque" id="29"/>
-    <tableColumn name="Recursos_captura" id="30"/>
-    <tableColumn name="Especies_importantes_captrura" id="31"/>
-    <tableColumn name="Destino" id="32"/>
-    <tableColumn name="Estado_comercializa_pescado" id="33"/>
-    <tableColumn name="Compra_produçao" id="34"/>
-    <tableColumn name="Preco_justo" id="35"/>
-    <tableColumn name="Problemas_comercializacao" id="36"/>
-    <tableColumn name="Cadastrado_organizacao" id="37"/>
-    <tableColumn name="Fatores_prejudicam_pesca" id="38"/>
-    <tableColumn name="Melhorias_TPLC" id="39"/>
-    <tableColumn name="Sugestao_TPLC" id="40"/>
-    <tableColumn name="Sugestao_mulheres_TPLC" id="41"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nome"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Comunidade"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Genero"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Idade"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Estado_civil"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Contato"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Numero_dependentes_renda"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Familia_escolaridade"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Familia_faixa_etaria"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Renda_mensal_total_familia"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Renda_origem"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Tipo_pesca"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Tempo_pesca(anos)"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Arte_pesca"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Duracao_pescaria"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Frequencia_pescaria"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Numero_tripulantes"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Pesca_defeso"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Seguro_defeso"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Embarcacao_propria"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Tipo_embarcaçao"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Porte_embarcacao"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Tipo_propulsao"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Dias_sem_reabastecer"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Titularidade"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Onde_pesca"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Local_saida"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Local_desenbarque"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Recursos_captura"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Especies_importantes_captrura"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Destino"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Estado_comercializa_pescado"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Compra_produçao"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Preco_justo"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Problemas_comercializacao"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Cadastrado_organizacao"/>
+    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Fatores_prejudicam_pesca"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Melhorias_TPLC"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Sugestao_TPLC"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Sugestao_mulheres_TPLC"/>
   </tableColumns>
-  <tableStyleInfo name="Página1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Página1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1137,29 +1147,32 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AO35"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="22.63"/>
-    <col customWidth="1" min="2" max="2" width="25.75"/>
-    <col customWidth="1" min="3" max="7" width="22.63"/>
-    <col customWidth="1" min="8" max="8" width="26.88"/>
-    <col customWidth="1" min="9" max="9" width="21.25"/>
-    <col customWidth="1" min="10" max="10" width="20.25"/>
-    <col customWidth="1" min="11" max="11" width="26.38"/>
-    <col customWidth="1" min="15" max="15" width="16.5"/>
-    <col customWidth="1" min="16" max="16" width="18.88"/>
-    <col customWidth="1" min="31" max="41" width="29.0"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="7" width="22.5703125" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="21.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20.28515625" customWidth="1"/>
+    <col min="11" max="11" width="26.42578125" customWidth="1"/>
+    <col min="15" max="15" width="16.42578125" customWidth="1"/>
+    <col min="16" max="16" width="18.85546875" customWidth="1"/>
+    <col min="31" max="41" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1284,9 +1297,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>41</v>
@@ -1304,10 +1317,10 @@
         <v>45</v>
       </c>
       <c r="G2" s="3">
-        <v>9.4223904E7</v>
+        <v>94223904</v>
       </c>
       <c r="H2" s="3">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>46</v>
@@ -1325,7 +1338,7 @@
         <v>50</v>
       </c>
       <c r="N2" s="3">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>51</v>
@@ -1337,7 +1350,7 @@
         <v>53</v>
       </c>
       <c r="R2" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>54</v>
@@ -1358,7 +1371,7 @@
         <v>58</v>
       </c>
       <c r="Y2" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="AA2" s="3" t="s">
         <v>59</v>
@@ -1404,9 +1417,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>71</v>
@@ -1424,10 +1437,10 @@
         <v>73</v>
       </c>
       <c r="G3" s="3">
-        <v>9.4814465E7</v>
+        <v>94814465</v>
       </c>
       <c r="H3" s="3">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>74</v>
@@ -1445,7 +1458,7 @@
         <v>50</v>
       </c>
       <c r="N3" s="3">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>78</v>
@@ -1457,7 +1470,7 @@
         <v>79</v>
       </c>
       <c r="R3" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>55</v>
@@ -1514,9 +1527,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>86</v>
@@ -1535,7 +1548,7 @@
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>46</v>
@@ -1550,7 +1563,7 @@
         <v>50</v>
       </c>
       <c r="N4" s="3">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>89</v>
@@ -1562,7 +1575,7 @@
         <v>53</v>
       </c>
       <c r="R4" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S4" s="3" t="s">
         <v>55</v>
@@ -1613,9 +1626,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>95</v>
@@ -1632,7 +1645,7 @@
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="3">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>96</v>
@@ -1650,7 +1663,7 @@
         <v>50</v>
       </c>
       <c r="N5" s="3">
-        <v>41.0</v>
+        <v>41</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>98</v>
@@ -1662,7 +1675,7 @@
         <v>53</v>
       </c>
       <c r="R5" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S5" s="3" t="s">
         <v>55</v>
@@ -1722,9 +1735,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>105</v>
@@ -1740,10 +1753,10 @@
         <v>45</v>
       </c>
       <c r="G6" s="3">
-        <v>9.9587556E8</v>
+        <v>995875560</v>
       </c>
       <c r="H6" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>106</v>
@@ -1761,7 +1774,7 @@
         <v>50</v>
       </c>
       <c r="N6" s="3">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>107</v>
@@ -1773,7 +1786,7 @@
         <v>53</v>
       </c>
       <c r="R6" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="S6" s="3" t="s">
         <v>55</v>
@@ -1833,9 +1846,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>116</v>
@@ -1854,7 +1867,7 @@
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>106</v>
@@ -1872,7 +1885,7 @@
         <v>50</v>
       </c>
       <c r="N7" s="3">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>119</v>
@@ -1884,7 +1897,7 @@
         <v>121</v>
       </c>
       <c r="R7" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S7" s="3" t="s">
         <v>55</v>
@@ -1950,9 +1963,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>128</v>
@@ -1969,7 +1982,7 @@
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>129</v>
@@ -1987,7 +2000,7 @@
         <v>50</v>
       </c>
       <c r="N8" s="3">
-        <v>45.0</v>
+        <v>45</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>119</v>
@@ -1999,7 +2012,7 @@
         <v>53</v>
       </c>
       <c r="R8" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S8" s="3" t="s">
         <v>55</v>
@@ -2068,9 +2081,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>136</v>
@@ -2087,7 +2100,7 @@
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>46</v>
@@ -2105,7 +2118,7 @@
         <v>50</v>
       </c>
       <c r="N9" s="3">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>137</v>
@@ -2117,7 +2130,7 @@
         <v>79</v>
       </c>
       <c r="R9" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S9" s="3" t="s">
         <v>55</v>
@@ -2138,7 +2151,7 @@
         <v>58</v>
       </c>
       <c r="Y9" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="Z9" s="3" t="s">
         <v>80</v>
@@ -2189,9 +2202,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>143</v>
@@ -2209,10 +2222,10 @@
         <v>73</v>
       </c>
       <c r="G10" s="3">
-        <v>9.4973276E7</v>
+        <v>94973276</v>
       </c>
       <c r="H10" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>74</v>
@@ -2230,7 +2243,7 @@
         <v>50</v>
       </c>
       <c r="N10" s="3">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>78</v>
@@ -2242,7 +2255,7 @@
         <v>53</v>
       </c>
       <c r="R10" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S10" s="3" t="s">
         <v>55</v>
@@ -2299,9 +2312,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>149</v>
@@ -2317,10 +2330,10 @@
         <v>45</v>
       </c>
       <c r="G11" s="3">
-        <v>9.4090391E7</v>
+        <v>94090391</v>
       </c>
       <c r="H11" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>74</v>
@@ -2338,7 +2351,7 @@
         <v>50</v>
       </c>
       <c r="N11" s="3">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>89</v>
@@ -2350,7 +2363,7 @@
         <v>79</v>
       </c>
       <c r="R11" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S11" s="3" t="s">
         <v>55</v>
@@ -2371,7 +2384,7 @@
         <v>151</v>
       </c>
       <c r="Y11" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="AA11" s="3" t="s">
         <v>59</v>
@@ -2416,9 +2429,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>154</v>
@@ -2436,10 +2449,10 @@
         <v>45</v>
       </c>
       <c r="G12" s="3">
-        <v>8.8744047E7</v>
+        <v>88744047</v>
       </c>
       <c r="H12" s="3">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>129</v>
@@ -2457,7 +2470,7 @@
         <v>50</v>
       </c>
       <c r="N12" s="3">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="O12" s="3" t="s">
         <v>89</v>
@@ -2469,7 +2482,7 @@
         <v>79</v>
       </c>
       <c r="R12" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S12" s="3" t="s">
         <v>54</v>
@@ -2490,7 +2503,7 @@
         <v>151</v>
       </c>
       <c r="Y12" s="3">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="AA12" s="3" t="s">
         <v>123</v>
@@ -2538,9 +2551,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>160</v>
@@ -2559,7 +2572,7 @@
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>74</v>
@@ -2577,7 +2590,7 @@
         <v>50</v>
       </c>
       <c r="N13" s="3">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="O13" s="3" t="s">
         <v>119</v>
@@ -2640,9 +2653,9 @@
         <v>164</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>165</v>
@@ -2660,10 +2673,10 @@
         <v>45</v>
       </c>
       <c r="G14" s="3">
-        <v>9.5087748E7</v>
+        <v>95087748</v>
       </c>
       <c r="H14" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>106</v>
@@ -2681,7 +2694,7 @@
         <v>50</v>
       </c>
       <c r="N14" s="3">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="O14" s="3" t="s">
         <v>137</v>
@@ -2693,7 +2706,7 @@
         <v>79</v>
       </c>
       <c r="R14" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S14" s="3" t="s">
         <v>55</v>
@@ -2714,7 +2727,7 @@
         <v>58</v>
       </c>
       <c r="Y14" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="AA14" s="3" t="s">
         <v>168</v>
@@ -2762,9 +2775,9 @@
         <v>174</v>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>175</v>
@@ -2782,10 +2795,10 @@
         <v>73</v>
       </c>
       <c r="G15" s="3">
-        <v>9.4295569E7</v>
+        <v>94295569</v>
       </c>
       <c r="H15" s="3">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>106</v>
@@ -2803,7 +2816,7 @@
         <v>50</v>
       </c>
       <c r="N15" s="3">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="O15" s="3" t="s">
         <v>119</v>
@@ -2815,7 +2828,7 @@
         <v>53</v>
       </c>
       <c r="R15" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S15" s="3" t="s">
         <v>55</v>
@@ -2836,7 +2849,7 @@
         <v>58</v>
       </c>
       <c r="Y15" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Z15" s="3" t="s">
         <v>108</v>
@@ -2887,9 +2900,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>178</v>
@@ -2907,10 +2920,10 @@
         <v>45</v>
       </c>
       <c r="G16" s="3">
-        <v>9.4521068E7</v>
+        <v>94521068</v>
       </c>
       <c r="H16" s="3">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>46</v>
@@ -2928,7 +2941,7 @@
         <v>50</v>
       </c>
       <c r="N16" s="3">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="O16" s="3" t="s">
         <v>180</v>
@@ -2940,7 +2953,7 @@
         <v>53</v>
       </c>
       <c r="R16" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S16" s="3" t="s">
         <v>55</v>
@@ -2961,7 +2974,7 @@
         <v>58</v>
       </c>
       <c r="Y16" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AA16" s="3" t="s">
         <v>59</v>
@@ -3009,9 +3022,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>187</v>
@@ -3030,7 +3043,7 @@
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="3">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>129</v>
@@ -3048,7 +3061,7 @@
         <v>50</v>
       </c>
       <c r="N17" s="3">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="O17" s="3" t="s">
         <v>78</v>
@@ -3060,7 +3073,7 @@
         <v>79</v>
       </c>
       <c r="R17" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S17" s="3" t="s">
         <v>55</v>
@@ -3081,7 +3094,7 @@
         <v>58</v>
       </c>
       <c r="Y17" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="AA17" s="3" t="s">
         <v>91</v>
@@ -3120,9 +3133,9 @@
         <v>191</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>192</v>
@@ -3140,10 +3153,10 @@
         <v>194</v>
       </c>
       <c r="G18" s="3">
-        <v>9.88126992E8</v>
+        <v>988126992</v>
       </c>
       <c r="H18" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>96</v>
@@ -3161,19 +3174,19 @@
         <v>50</v>
       </c>
       <c r="N18" s="3">
-        <v>48.0</v>
+        <v>48</v>
       </c>
       <c r="O18" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="P18" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="P18" s="3" t="s">
-        <v>197</v>
       </c>
       <c r="Q18" s="3" t="s">
         <v>79</v>
       </c>
       <c r="R18" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S18" s="3" t="s">
         <v>55</v>
@@ -3206,7 +3219,7 @@
         <v>61</v>
       </c>
       <c r="AE18" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AF18" s="3" t="s">
         <v>63</v>
@@ -3227,24 +3240,24 @@
         <v>112</v>
       </c>
       <c r="AL18" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AM18" s="3" t="s">
         <v>164</v>
       </c>
       <c r="AN18" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AO18" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="3" t="s">
@@ -3257,10 +3270,10 @@
         <v>45</v>
       </c>
       <c r="G19" s="3">
-        <v>9.5342603E7</v>
+        <v>95342603</v>
       </c>
       <c r="H19" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>106</v>
@@ -3275,19 +3288,19 @@
         <v>50</v>
       </c>
       <c r="N19" s="3">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="O19" s="3" t="s">
         <v>98</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Q19" s="3" t="s">
         <v>79</v>
       </c>
       <c r="R19" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S19" s="3" t="s">
         <v>55</v>
@@ -3305,10 +3318,10 @@
         <v>57</v>
       </c>
       <c r="X19" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Y19" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="Z19" s="3" t="s">
         <v>80</v>
@@ -3326,7 +3339,7 @@
         <v>61</v>
       </c>
       <c r="AE19" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AF19" s="3" t="s">
         <v>82</v>
@@ -3347,7 +3360,7 @@
         <v>94</v>
       </c>
       <c r="AM19" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AN19" s="3" t="s">
         <v>135</v>
@@ -3356,12 +3369,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
+    <row r="20" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>60</v>
@@ -3376,10 +3389,10 @@
         <v>73</v>
       </c>
       <c r="G20" s="3">
-        <v>9.94265055E8</v>
+        <v>994265055</v>
       </c>
       <c r="H20" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>74</v>
@@ -3394,19 +3407,19 @@
         <v>50</v>
       </c>
       <c r="N20" s="3">
-        <v>45.0</v>
+        <v>45</v>
       </c>
       <c r="O20" s="3" t="s">
         <v>78</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Q20" s="3" t="s">
         <v>53</v>
       </c>
       <c r="R20" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S20" s="3" t="s">
         <v>55</v>
@@ -3433,7 +3446,7 @@
         <v>61</v>
       </c>
       <c r="AE20" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AF20" s="3" t="s">
         <v>63</v>
@@ -3451,7 +3464,7 @@
         <v>112</v>
       </c>
       <c r="AL20" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="AM20" s="3" t="s">
         <v>147</v>
@@ -3463,12 +3476,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
+    <row r="21" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>60</v>
@@ -3484,10 +3497,10 @@
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="3">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>161</v>
@@ -3499,7 +3512,7 @@
         <v>50</v>
       </c>
       <c r="N21" s="3">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="O21" s="3" t="s">
         <v>137</v>
@@ -3511,7 +3524,7 @@
         <v>79</v>
       </c>
       <c r="R21" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S21" s="3" t="s">
         <v>55</v>
@@ -3532,7 +3545,7 @@
         <v>58</v>
       </c>
       <c r="Y21" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="AA21" s="3" t="s">
         <v>91</v>
@@ -3544,7 +3557,7 @@
         <v>61</v>
       </c>
       <c r="AE21" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AF21" s="3" t="s">
         <v>170</v>
@@ -3568,18 +3581,18 @@
         <v>134</v>
       </c>
       <c r="AN21" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AO21" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="22" ht="22.5" customHeight="1">
+    <row r="22" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>60</v>
@@ -3595,13 +3608,13 @@
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="3">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>46</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>77</v>
@@ -3619,7 +3632,7 @@
         <v>79</v>
       </c>
       <c r="R22" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S22" s="3" t="s">
         <v>55</v>
@@ -3640,7 +3653,7 @@
         <v>58</v>
       </c>
       <c r="Y22" s="3">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="AA22" s="3" t="s">
         <v>59</v>
@@ -3655,7 +3668,7 @@
         <v>61</v>
       </c>
       <c r="AE22" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AF22" s="3" t="s">
         <v>63</v>
@@ -3670,24 +3683,24 @@
         <v>55</v>
       </c>
       <c r="AL22" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="AM22" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="AM22" s="3" t="s">
+      <c r="AN22" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="AN22" s="3" t="s">
-        <v>219</v>
       </c>
       <c r="AO22" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="23" ht="22.5" customHeight="1">
+    <row r="23" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>60</v>
@@ -3703,10 +3716,10 @@
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>97</v>
@@ -3718,7 +3731,7 @@
         <v>50</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>138</v>
@@ -3727,7 +3740,7 @@
         <v>79</v>
       </c>
       <c r="R23" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S23" s="3" t="s">
         <v>54</v>
@@ -3748,7 +3761,7 @@
         <v>58</v>
       </c>
       <c r="Y23" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="AA23" s="3" t="s">
         <v>91</v>
@@ -3763,7 +3776,7 @@
         <v>61</v>
       </c>
       <c r="AE23" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AF23" s="3" t="s">
         <v>82</v>
@@ -3772,7 +3785,7 @@
         <v>64</v>
       </c>
       <c r="AH23" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AI23" s="3" t="s">
         <v>54</v>
@@ -3787,12 +3800,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="24" ht="22.5" customHeight="1">
+    <row r="24" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="3" t="s">
@@ -3806,7 +3819,7 @@
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>129</v>
@@ -3815,7 +3828,7 @@
         <v>47</v>
       </c>
       <c r="K24" s="3">
-        <v>500.0</v>
+        <v>500</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>88</v>
@@ -3824,7 +3837,7 @@
         <v>50</v>
       </c>
       <c r="N24" s="3">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="O24" s="3" t="s">
         <v>98</v>
@@ -3836,7 +3849,7 @@
         <v>53</v>
       </c>
       <c r="R24" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="S24" s="3" t="s">
         <v>55</v>
@@ -3857,7 +3870,7 @@
         <v>58</v>
       </c>
       <c r="Y24" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Z24" s="3" t="s">
         <v>108</v>
@@ -3875,7 +3888,7 @@
         <v>61</v>
       </c>
       <c r="AE24" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AF24" s="3" t="s">
         <v>63</v>
@@ -3890,7 +3903,7 @@
         <v>54</v>
       </c>
       <c r="AJ24" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AK24" s="3" t="s">
         <v>83</v>
@@ -3899,12 +3912,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" ht="22.5" customHeight="1">
+    <row r="25" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>60</v>
@@ -3920,7 +3933,7 @@
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="3">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>129</v>
@@ -3938,7 +3951,7 @@
         <v>50</v>
       </c>
       <c r="N25" s="3">
-        <v>44.0</v>
+        <v>44</v>
       </c>
       <c r="O25" s="3" t="s">
         <v>89</v>
@@ -3950,7 +3963,7 @@
         <v>79</v>
       </c>
       <c r="R25" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S25" s="3" t="s">
         <v>55</v>
@@ -3968,10 +3981,10 @@
         <v>57</v>
       </c>
       <c r="X25" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Y25" s="3">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="Z25" s="3" t="s">
         <v>108</v>
@@ -3989,7 +4002,7 @@
         <v>61</v>
       </c>
       <c r="AE25" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AF25" s="3" t="s">
         <v>63</v>
@@ -4004,7 +4017,7 @@
         <v>125</v>
       </c>
       <c r="AJ25" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AK25" s="3" t="s">
         <v>83</v>
@@ -4016,18 +4029,18 @@
         <v>172</v>
       </c>
       <c r="AN25" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AO25" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
+    <row r="26" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>60</v>
@@ -4043,7 +4056,7 @@
       </c>
       <c r="G26" s="4"/>
       <c r="H26" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>106</v>
@@ -4055,13 +4068,13 @@
         <v>97</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>50</v>
       </c>
       <c r="N26" s="3">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="O26" s="3" t="s">
         <v>89</v>
@@ -4073,7 +4086,7 @@
         <v>79</v>
       </c>
       <c r="R26" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S26" s="3" t="s">
         <v>55</v>
@@ -4091,10 +4104,10 @@
         <v>189</v>
       </c>
       <c r="X26" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Y26" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="AA26" s="3" t="s">
         <v>91</v>
@@ -4109,7 +4122,7 @@
         <v>61</v>
       </c>
       <c r="AE26" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AF26" s="3" t="s">
         <v>82</v>
@@ -4121,7 +4134,7 @@
         <v>65</v>
       </c>
       <c r="AL26" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AM26" s="3" t="s">
         <v>84</v>
@@ -4130,12 +4143,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
+    <row r="27" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>42</v>
@@ -4150,10 +4163,10 @@
         <v>45</v>
       </c>
       <c r="G27" s="3">
-        <v>8.694166062E9</v>
+        <v>8694166062</v>
       </c>
       <c r="H27" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>106</v>
@@ -4171,7 +4184,7 @@
         <v>50</v>
       </c>
       <c r="N27" s="3">
-        <v>40.0</v>
+        <v>40</v>
       </c>
       <c r="O27" s="3" t="s">
         <v>119</v>
@@ -4183,7 +4196,7 @@
         <v>53</v>
       </c>
       <c r="R27" s="3">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="S27" s="3" t="s">
         <v>55</v>
@@ -4201,13 +4214,13 @@
         <v>189</v>
       </c>
       <c r="X27" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y27" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA27" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="Y27" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="AA27" s="3" t="s">
-        <v>237</v>
       </c>
       <c r="AB27" s="3" t="s">
         <v>60</v>
@@ -4219,7 +4232,7 @@
         <v>61</v>
       </c>
       <c r="AE27" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AF27" s="3" t="s">
         <v>63</v>
@@ -4240,18 +4253,18 @@
         <v>84</v>
       </c>
       <c r="AN27" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AO27" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="28" ht="22.5" customHeight="1">
+    <row r="28" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>60</v>
@@ -4267,7 +4280,7 @@
       </c>
       <c r="G28" s="4"/>
       <c r="H28" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>74</v>
@@ -4282,7 +4295,7 @@
         <v>50</v>
       </c>
       <c r="N28" s="3">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="O28" s="3" t="s">
         <v>89</v>
@@ -4294,7 +4307,7 @@
         <v>79</v>
       </c>
       <c r="R28" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S28" s="3" t="s">
         <v>55</v>
@@ -4309,7 +4322,7 @@
         <v>80</v>
       </c>
       <c r="AA28" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AB28" s="3" t="s">
         <v>60</v>
@@ -4339,21 +4352,21 @@
         <v>66</v>
       </c>
       <c r="AL28" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AM28" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AO28" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" ht="22.5" customHeight="1">
+    <row r="29" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>60</v>
@@ -4369,10 +4382,10 @@
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>47</v>
@@ -4387,7 +4400,7 @@
         <v>50</v>
       </c>
       <c r="N29" s="3">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="O29" s="3" t="s">
         <v>89</v>
@@ -4399,7 +4412,7 @@
         <v>53</v>
       </c>
       <c r="R29" s="3">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="S29" s="3" t="s">
         <v>55</v>
@@ -4417,13 +4430,13 @@
         <v>57</v>
       </c>
       <c r="X29" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA29" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="Y29" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="AA29" s="3" t="s">
-        <v>237</v>
       </c>
       <c r="AB29" s="3" t="s">
         <v>60</v>
@@ -4435,7 +4448,7 @@
         <v>61</v>
       </c>
       <c r="AE29" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AF29" s="3" t="s">
         <v>63</v>
@@ -4459,18 +4472,18 @@
         <v>84</v>
       </c>
       <c r="AN29" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AO29" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="30" ht="22.5" customHeight="1">
+    <row r="30" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="3" t="s">
@@ -4484,16 +4497,16 @@
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J30" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="K30" s="3" t="s">
         <v>245</v>
-      </c>
-      <c r="K30" s="3" t="s">
-        <v>246</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>88</v>
@@ -4502,7 +4515,7 @@
         <v>50</v>
       </c>
       <c r="N30" s="3">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="O30" s="3" t="s">
         <v>78</v>
@@ -4514,7 +4527,7 @@
         <v>79</v>
       </c>
       <c r="R30" s="3">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="S30" s="3" t="s">
         <v>55</v>
@@ -4535,13 +4548,13 @@
         <v>58</v>
       </c>
       <c r="Y30" s="3">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Z30" s="3" t="s">
         <v>80</v>
       </c>
       <c r="AA30" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AB30" s="3" t="s">
         <v>60</v>
@@ -4553,10 +4566,10 @@
         <v>182</v>
       </c>
       <c r="AE30" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="AF30" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="AF30" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="AG30" s="3" t="s">
         <v>64</v>
@@ -4568,22 +4581,22 @@
         <v>54</v>
       </c>
       <c r="AJ30" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AL30" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AM30" s="3" t="s">
         <v>84</v>
       </c>
       <c r="AN30" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AO30" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="31" ht="22.5" customHeight="1">
+    <row r="31" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -4592,7 +4605,7 @@
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
     </row>
-    <row r="32" ht="22.5" customHeight="1">
+    <row r="32" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -4601,7 +4614,7 @@
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" ht="22.5" customHeight="1">
+    <row r="33" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -4610,7 +4623,7 @@
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" ht="22.5" customHeight="1">
+    <row r="34" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -4619,7 +4632,7 @@
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
     </row>
-    <row r="35" ht="22.5" customHeight="1">
+    <row r="35" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -4629,9 +4642,9 @@
       <c r="G35" s="4"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>